<commit_message>
feat: update for business logic & new graphics
</commit_message>
<xml_diff>
--- a/public/templates/template_update_sku.xlsx
+++ b/public/templates/template_update_sku.xlsx
@@ -401,10 +401,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>old_hemicode</v>
+        <v>old_cn_code</v>
       </c>
       <c r="B1" t="str">
-        <v>new_hemicode</v>
+        <v>new_cn_code</v>
       </c>
     </row>
     <row r="2">

</xml_diff>